<commit_message>
I made some changes to the faculty data and it is now fully ready to be imported into the data base
</commit_message>
<xml_diff>
--- a/Faculties/Natural Science/Programmes Natural Science.xlsx
+++ b/Faculties/Natural Science/Programmes Natural Science.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d24d4a286855a075/Desktop/Team_6_repo/Team19/Faculties/Natural Science/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="11_F25DC773A252ABDACC10480281DB6CA25BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F917FCCF-0A6B-443A-828D-A89C76206B0C}"/>
+  <xr:revisionPtr revIDLastSave="79" documentId="11_F25DC773A252ABDACC10480281DB6CA25BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94ED27CA-EDE0-4632-A4A2-85DE96DA9024}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,265 +36,265 @@
     <t>Abbreviation</t>
   </si>
   <si>
-    <t>BSc (Applied Geology)</t>
-  </si>
-  <si>
-    <t>BSc (Biodiversity and Conservation Biology)</t>
-  </si>
-  <si>
-    <t>BSc (Biotechnology)</t>
-  </si>
-  <si>
-    <t>BSc (Chemical Sciences)</t>
-  </si>
-  <si>
-    <t>BSc (Computer Science)</t>
-  </si>
-  <si>
-    <t>BSc (Environment and Water Science)</t>
-  </si>
-  <si>
-    <t>BSc (Mathematics and Statistical Sciences)</t>
-  </si>
-  <si>
-    <t>BSc (Medical Bioscience)</t>
-  </si>
-  <si>
-    <t>BSc (Physical Science)</t>
-  </si>
-  <si>
     <t>BPharm</t>
   </si>
   <si>
-    <t>BScHons (Applied Geology)</t>
-  </si>
-  <si>
-    <t>BScHons (Astrophysics)</t>
-  </si>
-  <si>
-    <t>BScHons (Biodiversity and Conservation Biology)</t>
-  </si>
-  <si>
-    <t>BScHons (Biotechnology)</t>
-  </si>
-  <si>
-    <t>BScHons (Chemistry)</t>
-  </si>
-  <si>
-    <t>BScHons (Computational Finance)</t>
-  </si>
-  <si>
-    <t>BScHons (Computer Science)</t>
-  </si>
-  <si>
-    <t>BScHons (Environment and Water Science)</t>
-  </si>
-  <si>
-    <t>BScHons (Mathematics)</t>
-  </si>
-  <si>
-    <t>BScHons (Medical Bioscience)</t>
-  </si>
-  <si>
-    <t>BScHons (Physical Science)</t>
-  </si>
-  <si>
-    <t>BScHons (Population Studies)</t>
-  </si>
-  <si>
-    <t>BScHons (Statistical Science)</t>
-  </si>
-  <si>
     <t>MPharm</t>
   </si>
   <si>
-    <t>MPhil (Population Studies)</t>
-  </si>
-  <si>
-    <t>MSc (Applied Geology)</t>
-  </si>
-  <si>
-    <t>MSc (Biodiversity and Conservation Biology)</t>
-  </si>
-  <si>
-    <t>MSc (Bioinformatics)</t>
-  </si>
-  <si>
-    <t>MSc (Biotechnology)</t>
-  </si>
-  <si>
-    <t>MSc (Chemical Sciences)</t>
-  </si>
-  <si>
-    <t>MSc (Computational Finance)</t>
-  </si>
-  <si>
-    <t>MSc (Computer Science)</t>
-  </si>
-  <si>
-    <t>MSc (Environment and Water Science)</t>
-  </si>
-  <si>
-    <t>Duration (Years)</t>
-  </si>
-  <si>
-    <t>1. Bachelor of Science in Applied Geology</t>
-  </si>
-  <si>
-    <t>2. Bachelor of Science in Biodiversity and Conservation Biology</t>
-  </si>
-  <si>
-    <t>3. Bachelor of Science in Biotechnology</t>
-  </si>
-  <si>
-    <t>4. Bachelor of Science in Chemical Sciences</t>
-  </si>
-  <si>
-    <t>5. Bachelor of Science in Computer Science</t>
-  </si>
-  <si>
-    <t>6. Bachelor of Science in Environment and Water Science</t>
-  </si>
-  <si>
-    <t>7. Bachelor of Science in Mathematics and Statistical Sciences</t>
-  </si>
-  <si>
-    <t>8. Bachelor of Science in Medical Bioscience</t>
-  </si>
-  <si>
-    <t>9. Bachelor of Science in Physical Science</t>
-  </si>
-  <si>
-    <t>10. Bachelor of Pharmacy</t>
-  </si>
-  <si>
-    <t>11. Bachelor of Science Honours in Applied Geology</t>
-  </si>
-  <si>
-    <t>12. Bachelor of Science Honours in Astrophysics</t>
-  </si>
-  <si>
-    <t>13. Bachelor of Science Honours in Biodiversity and Conservation Biology</t>
-  </si>
-  <si>
-    <t>14. Bachelor of Science Honours in Biotechnology</t>
-  </si>
-  <si>
-    <t>15. Bachelor of Science Honours in Chemistry</t>
-  </si>
-  <si>
-    <t>16. Bachelor of Science Honours in Computational Finance</t>
-  </si>
-  <si>
-    <t>17. Bachelor of Science Honours in Computer Science</t>
-  </si>
-  <si>
-    <t>18. Bachelor of Science Honours in Environment and Water Science</t>
-  </si>
-  <si>
-    <t>19. Bachelor of Science Honours in Mathematics</t>
-  </si>
-  <si>
-    <t>20. Bachelor of Science Honours in Medical Bioscience</t>
-  </si>
-  <si>
-    <t>21. Bachelor of Science Honours in Physical Science</t>
-  </si>
-  <si>
-    <t>22. Bachelor of Science Honours in Population Studies</t>
-  </si>
-  <si>
-    <t>23. Bachelor of Science Honours in Statistical Science</t>
-  </si>
-  <si>
-    <t>24. Master of Pharmacy</t>
-  </si>
-  <si>
-    <t>25. Master of Philosophy in Population Studies</t>
-  </si>
-  <si>
-    <t>26. Master of Science in Applied Geology</t>
-  </si>
-  <si>
-    <t>27. Master of Science in Biodiversity and Conservation Biology</t>
-  </si>
-  <si>
-    <t>28. Master of Science in Bioinformatics</t>
-  </si>
-  <si>
-    <t>29. Master of Science in Biotechnology</t>
-  </si>
-  <si>
-    <t>30. Master of Science in Chemical Sciences</t>
-  </si>
-  <si>
-    <t>31. Master of Science in Computational Finance</t>
-  </si>
-  <si>
-    <t>32. Master of Science in Computer Science</t>
-  </si>
-  <si>
-    <t>33. Master of Science in Environment and Water Science</t>
-  </si>
-  <si>
-    <t>34. Master of Science in Mathematical Science</t>
-  </si>
-  <si>
-    <t>MSc (Mathematical Science)</t>
-  </si>
-  <si>
-    <t>35. Master of Science in Medical Bioscience</t>
-  </si>
-  <si>
-    <t>MSc (Medical Bioscience)</t>
-  </si>
-  <si>
-    <t>36. Master of Science in Nanoscience</t>
-  </si>
-  <si>
-    <t>MSc (Nanoscience)</t>
-  </si>
-  <si>
-    <t>37. Master of Science in Pharmaceutical Sciences</t>
-  </si>
-  <si>
-    <t>MSc (Pharmaceutical Sciences)</t>
-  </si>
-  <si>
-    <t>38. Master of Science in Pharmacy Administration and Policy Regulation</t>
-  </si>
-  <si>
-    <t>MSc (Pharmacy Administration and Policy Regulation)</t>
-  </si>
-  <si>
-    <t>39. Master of Science in Physical Science</t>
-  </si>
-  <si>
-    <t>MSc (Physical Science)</t>
-  </si>
-  <si>
-    <t>40. Master of Science in Statistical Science</t>
-  </si>
-  <si>
-    <t>MSc (Statistical Science)</t>
-  </si>
-  <si>
-    <t>41. Master of Clinical Pharmacy</t>
-  </si>
-  <si>
     <t>M Clinical Pharmacy</t>
   </si>
   <si>
-    <t>42. Doctor of Pharmacy</t>
-  </si>
-  <si>
     <t>DPharm</t>
   </si>
   <si>
-    <t>43. Doctor of Philosophy</t>
-  </si>
-  <si>
     <t>PhD</t>
+  </si>
+  <si>
+    <t>Bachelor of Science in Applied Geology</t>
+  </si>
+  <si>
+    <t>Bachelor of Science in Biodiversity and Conservation Biology</t>
+  </si>
+  <si>
+    <t>Bachelor of Science in Biotechnology</t>
+  </si>
+  <si>
+    <t>Bachelor of Science in Chemical Sciences</t>
+  </si>
+  <si>
+    <t>Bachelor of Science in Computer Science</t>
+  </si>
+  <si>
+    <t>Bachelor of Science in Environment and Water Science</t>
+  </si>
+  <si>
+    <t>Bachelor of Science in Mathematics and Statistical Sciences</t>
+  </si>
+  <si>
+    <t>Bachelor of Science in Medical Bioscience</t>
+  </si>
+  <si>
+    <t>Bachelor of Science in Physical Science</t>
+  </si>
+  <si>
+    <t>Bachelor of Pharmacy</t>
+  </si>
+  <si>
+    <t>Bachelor of Science Honours in Applied Geology</t>
+  </si>
+  <si>
+    <t>Bachelor of Science Honours in Astrophysics</t>
+  </si>
+  <si>
+    <t>Bachelor of Science Honours in Biodiversity and Conservation Biology</t>
+  </si>
+  <si>
+    <t>Bachelor of Science Honours in Biotechnology</t>
+  </si>
+  <si>
+    <t>Bachelor of Science Honours in Chemistry</t>
+  </si>
+  <si>
+    <t>Bachelor of Science Honours in Computational Finance</t>
+  </si>
+  <si>
+    <t>Bachelor of Science Honours in Computer Science</t>
+  </si>
+  <si>
+    <t>Bachelor of Science Honours in Environment and Water Science</t>
+  </si>
+  <si>
+    <t>Bachelor of Science Honours in Mathematics</t>
+  </si>
+  <si>
+    <t>Bachelor of Science Honours in Medical Bioscience</t>
+  </si>
+  <si>
+    <t>Bachelor of Science Honours in Physical Science</t>
+  </si>
+  <si>
+    <t>Bachelor of Science Honours in Population Studies</t>
+  </si>
+  <si>
+    <t>Bachelor of Science Honours in Statistical Science</t>
+  </si>
+  <si>
+    <t>Master of Pharmacy</t>
+  </si>
+  <si>
+    <t>Master of Philosophy in Population Studies</t>
+  </si>
+  <si>
+    <t>Master of Science in Applied Geology</t>
+  </si>
+  <si>
+    <t>Master of Science in Biodiversity and Conservation Biology</t>
+  </si>
+  <si>
+    <t>Master of Science in Bioinformatics</t>
+  </si>
+  <si>
+    <t>Master of Science in Biotechnology</t>
+  </si>
+  <si>
+    <t>Master of Science in Chemical Sciences</t>
+  </si>
+  <si>
+    <t>Master of Science in Computational Finance</t>
+  </si>
+  <si>
+    <t>Master of Science in Computer Science</t>
+  </si>
+  <si>
+    <t>Master of Science in Environment and Water Science</t>
+  </si>
+  <si>
+    <t>Master of Science in Mathematical Science</t>
+  </si>
+  <si>
+    <t>Master of Science in Medical Bioscience</t>
+  </si>
+  <si>
+    <t>Master of Science in Nanoscience</t>
+  </si>
+  <si>
+    <t>Master of Science in Pharmaceutical Sciences</t>
+  </si>
+  <si>
+    <t>Master of Science in Pharmacy Administration and Policy Regulation</t>
+  </si>
+  <si>
+    <t>Master of Science in Physical Science</t>
+  </si>
+  <si>
+    <t>Master of Science in Statistical Science</t>
+  </si>
+  <si>
+    <t>Master of Clinical Pharmacy</t>
+  </si>
+  <si>
+    <t>Doctor of Pharmacy</t>
+  </si>
+  <si>
+    <t>Doctor of Philosophy</t>
+  </si>
+  <si>
+    <t>Duration  Years)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSc  Applied Geology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSc  Biodiversity and Conservation Biology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSc  Biotechnology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSc  Chemical Sciences </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSc  Computer Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSc  Environment and Water Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSc  Mathematics and Statistical Sciences </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSc  Medical Bioscience </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSc  Physical Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons  Applied Geology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons  Astrophysics </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons  Biodiversity and Conservation Biology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons  Biotechnology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons  Chemistry </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons  Computational Finance </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons  Computer Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons  Environment and Water Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons  Mathematics </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons  Medical Bioscience </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons  Physical Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons  Population Studies </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons  Statistical Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MPhil  Population Studies </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc  Applied Geology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc  Biodiversity and Conservation Biology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc  Bioinformatics </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc  Biotechnology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc  Chemical Sciences </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc  Computational Finance </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc  Computer Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc  Environment and Water Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc  Mathematical Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc  Medical Bioscience </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc  Nanoscience </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc  Pharmaceutical Sciences </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc  Pharmacy Administration and Policy Regulation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc  Physical Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc  Statistical Science </t>
   </si>
 </sst>
 </file>
@@ -366,6 +366,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -636,7 +640,7 @@
   <cols>
     <col min="1" max="1" width="18.5546875" customWidth="1"/>
     <col min="2" max="2" width="20.5546875" customWidth="1"/>
-    <col min="3" max="3" width="15.33203125" customWidth="1"/>
+    <col min="3" max="3" width="25.88671875" customWidth="1"/>
     <col min="4" max="4" width="18.5546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -651,18 +655,18 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="B2" s="2">
         <v>3214</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>3</v>
+        <v>52</v>
       </c>
       <c r="D2" s="2">
         <v>3</v>
@@ -670,13 +674,13 @@
     </row>
     <row r="3" spans="1:4" ht="78" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="B3" s="2">
         <v>3217</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>4</v>
+        <v>53</v>
       </c>
       <c r="D3" s="2">
         <v>3</v>
@@ -684,13 +688,13 @@
     </row>
     <row r="4" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="B4" s="2">
         <v>3211</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="D4" s="2">
         <v>3</v>
@@ -698,13 +702,13 @@
     </row>
     <row r="5" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="B5" s="2">
         <v>3220</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>6</v>
+        <v>55</v>
       </c>
       <c r="D5" s="2">
         <v>3</v>
@@ -712,13 +716,13 @@
     </row>
     <row r="6" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="B6" s="2">
         <v>3221</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>7</v>
+        <v>56</v>
       </c>
       <c r="D6" s="2">
         <v>3</v>
@@ -726,13 +730,13 @@
     </row>
     <row r="7" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="B7" s="2">
         <v>3331</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>8</v>
+        <v>57</v>
       </c>
       <c r="D7" s="2">
         <v>3</v>
@@ -740,13 +744,13 @@
     </row>
     <row r="8" spans="1:4" ht="78" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="B8" s="2">
         <v>3227</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="D8" s="2">
         <v>3</v>
@@ -754,13 +758,13 @@
     </row>
     <row r="9" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="B9" s="2">
         <v>3230</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>10</v>
+        <v>59</v>
       </c>
       <c r="D9" s="2">
         <v>3</v>
@@ -768,13 +772,13 @@
     </row>
     <row r="10" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="B10" s="2">
         <v>3233</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>11</v>
+        <v>60</v>
       </c>
       <c r="D10" s="2">
         <v>3</v>
@@ -782,13 +786,13 @@
     </row>
     <row r="11" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="B11" s="2">
         <v>3305</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D11" s="2">
         <v>4</v>
@@ -796,13 +800,13 @@
     </row>
     <row r="12" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>47</v>
+        <v>18</v>
       </c>
       <c r="B12" s="2">
         <v>3710</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>13</v>
+        <v>61</v>
       </c>
       <c r="D12" s="2">
         <v>1</v>
@@ -810,13 +814,13 @@
     </row>
     <row r="13" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>48</v>
+        <v>19</v>
       </c>
       <c r="B13" s="2">
         <v>3793</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="D13" s="2">
         <v>1</v>
@@ -824,13 +828,13 @@
     </row>
     <row r="14" spans="1:4" ht="78" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="B14" s="2">
         <v>3731</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>15</v>
+        <v>63</v>
       </c>
       <c r="D14" s="2">
         <v>1</v>
@@ -838,13 +842,13 @@
     </row>
     <row r="15" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="B15" s="2">
         <v>3707</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>16</v>
+        <v>64</v>
       </c>
       <c r="D15" s="2">
         <v>1</v>
@@ -852,13 +856,13 @@
     </row>
     <row r="16" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="B16" s="2">
         <v>3734</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>17</v>
+        <v>65</v>
       </c>
       <c r="D16" s="2">
         <v>1</v>
@@ -866,13 +870,13 @@
     </row>
     <row r="17" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="B17" s="2">
         <v>3739</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="D17" s="2">
         <v>1</v>
@@ -880,13 +884,13 @@
     </row>
     <row r="18" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="B18" s="2">
         <v>3735</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>19</v>
+        <v>67</v>
       </c>
       <c r="D18" s="2">
         <v>1</v>
@@ -894,13 +898,13 @@
     </row>
     <row r="19" spans="1:4" ht="78" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="B19" s="2">
         <v>3780</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="D19" s="2">
         <v>1</v>
@@ -908,13 +912,13 @@
     </row>
     <row r="20" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="B20" s="2">
         <v>3736</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>21</v>
+        <v>69</v>
       </c>
       <c r="D20" s="2">
         <v>1</v>
@@ -922,13 +926,13 @@
     </row>
     <row r="21" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="B21" s="2">
         <v>3721</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>22</v>
+        <v>70</v>
       </c>
       <c r="D21" s="2">
         <v>1</v>
@@ -936,13 +940,13 @@
     </row>
     <row r="22" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="B22" s="2">
         <v>3714</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="D22" s="2">
         <v>1</v>
@@ -950,13 +954,13 @@
     </row>
     <row r="23" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="B23" s="2">
         <v>3738</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="D23" s="2">
         <v>1</v>
@@ -964,13 +968,13 @@
     </row>
     <row r="24" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B24" s="2">
         <v>3737</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>25</v>
+        <v>73</v>
       </c>
       <c r="D24" s="2">
         <v>1</v>
@@ -978,13 +982,13 @@
     </row>
     <row r="25" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="B25" s="2">
         <v>3851</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="D25" s="2">
         <v>1</v>
@@ -992,13 +996,13 @@
     </row>
     <row r="26" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>61</v>
+        <v>32</v>
       </c>
       <c r="B26" s="2">
         <v>3921</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>27</v>
+        <v>74</v>
       </c>
       <c r="D26" s="2">
         <v>1</v>
@@ -1006,13 +1010,13 @@
     </row>
     <row r="27" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="B27" s="2">
         <v>3891</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>28</v>
+        <v>75</v>
       </c>
       <c r="D27" s="2">
         <v>1</v>
@@ -1020,83 +1024,83 @@
     </row>
     <row r="28" spans="1:4" ht="78" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="B28" s="2">
         <v>3824</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="D28" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="B29" s="2">
         <v>3895</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="D29" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="B30" s="2">
         <v>3185</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>31</v>
+        <v>78</v>
       </c>
       <c r="D30" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>66</v>
+        <v>37</v>
       </c>
       <c r="B31" s="2">
         <v>3823</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>32</v>
+        <v>79</v>
       </c>
       <c r="D31" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="B32" s="2">
         <v>3093</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>33</v>
+        <v>80</v>
       </c>
       <c r="D32" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="B33" s="2">
         <v>3848</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>34</v>
+        <v>81</v>
       </c>
       <c r="D33" s="2">
         <v>1</v>
@@ -1104,55 +1108,55 @@
     </row>
     <row r="34" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>69</v>
+        <v>40</v>
       </c>
       <c r="B34" s="2">
         <v>3085</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>35</v>
+        <v>82</v>
       </c>
       <c r="D34" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="B35" s="2">
         <v>3849</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="D35" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>72</v>
+        <v>42</v>
       </c>
       <c r="B36" s="2">
         <v>3819</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="D36" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>74</v>
+        <v>43</v>
       </c>
       <c r="B37" s="2">
         <v>3089</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="D37" s="2">
         <v>2</v>
@@ -1160,27 +1164,27 @@
     </row>
     <row r="38" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>76</v>
+        <v>44</v>
       </c>
       <c r="B38" s="2">
         <v>3181</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="D38" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="93.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" ht="78" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="B39" s="2">
         <v>3859</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="D39" s="2">
         <v>2</v>
@@ -1188,41 +1192,41 @@
     </row>
     <row r="40" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>80</v>
+        <v>46</v>
       </c>
       <c r="B40" s="2">
         <v>3081</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="D40" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>82</v>
+        <v>47</v>
       </c>
       <c r="B41" s="2">
         <v>3838</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="D41" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>84</v>
+        <v>48</v>
       </c>
       <c r="B42" s="2">
         <v>3852</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>85</v>
+        <v>5</v>
       </c>
       <c r="D42" s="2">
         <v>3</v>
@@ -1230,13 +1234,13 @@
     </row>
     <row r="43" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="B43" s="2">
         <v>3951</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>87</v>
+        <v>6</v>
       </c>
       <c r="D43" s="2">
         <v>2</v>
@@ -1244,13 +1248,13 @@
     </row>
     <row r="44" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>88</v>
+        <v>50</v>
       </c>
       <c r="B44" s="2">
         <v>3961</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>89</v>
+        <v>7</v>
       </c>
       <c r="D44" s="2">
         <v>2</v>

</xml_diff>

<commit_message>
I have created the course_insertion file as well as made an adjustment to my tech stack
</commit_message>
<xml_diff>
--- a/Faculties/Natural Science/Programmes Natural Science.xlsx
+++ b/Faculties/Natural Science/Programmes Natural Science.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d24d4a286855a075/Desktop/Team_6_repo/Team19/Faculties/Natural Science/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="80" documentId="11_F25DC773A252ABDACC10480281DB6CA25BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C709630-A496-4A0D-B909-98BA3136C022}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="11_F25DC773A252ABDACC10480281DB6CA25BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87AFA6C6-0336-441E-B7D1-D86345739998}"/>
   <bookViews>
-    <workbookView xWindow="10596" yWindow="708" windowWidth="9984" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12084" yWindow="2064" windowWidth="9984" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -180,121 +180,121 @@
     <t>Doctor of Philosophy</t>
   </si>
   <si>
-    <t xml:space="preserve">BSc  Applied Geology </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BSc  Biodiversity and Conservation Biology </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BSc  Biotechnology </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BSc  Chemical Sciences </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BSc  Computer Science </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BSc  Environment and Water Science </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BSc  Mathematics and Statistical Sciences </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BSc  Medical Bioscience </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BSc  Physical Science </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BScHons  Applied Geology </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BScHons  Astrophysics </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BScHons  Biodiversity and Conservation Biology </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BScHons  Biotechnology </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BScHons  Chemistry </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BScHons  Computational Finance </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BScHons  Computer Science </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BScHons  Environment and Water Science </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BScHons  Mathematics </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BScHons  Medical Bioscience </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BScHons  Physical Science </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BScHons  Population Studies </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BScHons  Statistical Science </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MPhil  Population Studies </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSc  Applied Geology </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSc  Biodiversity and Conservation Biology </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSc  Bioinformatics </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSc  Biotechnology </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSc  Chemical Sciences </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSc  Computational Finance </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSc  Computer Science </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSc  Environment and Water Science </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSc  Mathematical Science </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSc  Medical Bioscience </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSc  Nanoscience </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSc  Pharmaceutical Sciences </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSc  Pharmacy Administration and Policy Regulation </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSc  Physical Science </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSc  Statistical Science </t>
-  </si>
-  <si>
-    <t>Duration  Years</t>
+    <t>Duration Years</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSc Applied Geology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSc Biodiversity and Conservation Biology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSc Biotechnology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSc Chemical Sciences </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSc Computer Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSc Environment and Water Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSc Mathematics and Statistical Sciences </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSc Medical Bioscience </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSc Physical Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons Applied Geology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons Astrophysics </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons Biodiversity and Conservation Biology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons Biotechnology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons Chemistry </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons Computational Finance </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons Computer Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons Environment and Water Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons Mathematics </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons Medical Bioscience </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons Physical Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons Population Studies </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BScHons Statistical Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MPhil Population Studies </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc Applied Geology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc Biodiversity and Conservation Biology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc Bioinformatics </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc Biotechnology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc Chemical Sciences </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc Computational Finance </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc Computer Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc Environment and Water Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc Mathematical Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc Medical Bioscience </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc Nanoscience </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc Pharmaceutical Sciences </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc Pharmacy Administration and Policy Regulation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc Physical Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSc Statistical Science </t>
   </si>
 </sst>
 </file>
@@ -655,7 +655,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>89</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
@@ -666,7 +666,7 @@
         <v>3214</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D2" s="2">
         <v>3</v>
@@ -680,7 +680,7 @@
         <v>3217</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D3" s="2">
         <v>3</v>
@@ -694,7 +694,7 @@
         <v>3211</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D4" s="2">
         <v>3</v>
@@ -708,7 +708,7 @@
         <v>3220</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D5" s="2">
         <v>3</v>
@@ -722,7 +722,7 @@
         <v>3221</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D6" s="2">
         <v>3</v>
@@ -736,7 +736,7 @@
         <v>3331</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D7" s="2">
         <v>3</v>
@@ -750,7 +750,7 @@
         <v>3227</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D8" s="2">
         <v>3</v>
@@ -764,7 +764,7 @@
         <v>3230</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D9" s="2">
         <v>3</v>
@@ -778,7 +778,7 @@
         <v>3233</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D10" s="2">
         <v>3</v>
@@ -806,7 +806,7 @@
         <v>3710</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D12" s="2">
         <v>1</v>
@@ -820,7 +820,7 @@
         <v>3793</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D13" s="2">
         <v>1</v>
@@ -834,7 +834,7 @@
         <v>3731</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D14" s="2">
         <v>1</v>
@@ -848,7 +848,7 @@
         <v>3707</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D15" s="2">
         <v>1</v>
@@ -862,7 +862,7 @@
         <v>3734</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D16" s="2">
         <v>1</v>
@@ -876,7 +876,7 @@
         <v>3739</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D17" s="2">
         <v>1</v>
@@ -890,7 +890,7 @@
         <v>3735</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D18" s="2">
         <v>1</v>
@@ -904,7 +904,7 @@
         <v>3780</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D19" s="2">
         <v>1</v>
@@ -918,7 +918,7 @@
         <v>3736</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D20" s="2">
         <v>1</v>
@@ -932,7 +932,7 @@
         <v>3721</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D21" s="2">
         <v>1</v>
@@ -946,7 +946,7 @@
         <v>3714</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D22" s="2">
         <v>1</v>
@@ -960,7 +960,7 @@
         <v>3738</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D23" s="2">
         <v>1</v>
@@ -974,7 +974,7 @@
         <v>3737</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D24" s="2">
         <v>1</v>
@@ -1002,7 +1002,7 @@
         <v>3921</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D26" s="2">
         <v>1</v>
@@ -1016,7 +1016,7 @@
         <v>3891</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D27" s="2">
         <v>1</v>
@@ -1030,7 +1030,7 @@
         <v>3824</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D28" s="2">
         <v>1</v>
@@ -1044,7 +1044,7 @@
         <v>3895</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D29" s="2">
         <v>1</v>
@@ -1058,7 +1058,7 @@
         <v>3185</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D30" s="2">
         <v>1</v>
@@ -1072,7 +1072,7 @@
         <v>3823</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D31" s="2">
         <v>1</v>
@@ -1086,7 +1086,7 @@
         <v>3093</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D32" s="2">
         <v>1</v>
@@ -1100,7 +1100,7 @@
         <v>3848</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D33" s="2">
         <v>1</v>
@@ -1114,7 +1114,7 @@
         <v>3085</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D34" s="2">
         <v>1</v>
@@ -1128,7 +1128,7 @@
         <v>3849</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D35" s="2">
         <v>1</v>
@@ -1142,7 +1142,7 @@
         <v>3819</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D36" s="2">
         <v>1</v>
@@ -1156,7 +1156,7 @@
         <v>3089</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D37" s="2">
         <v>2</v>
@@ -1170,7 +1170,7 @@
         <v>3181</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D38" s="2">
         <v>2</v>
@@ -1184,7 +1184,7 @@
         <v>3859</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D39" s="2">
         <v>2</v>
@@ -1198,7 +1198,7 @@
         <v>3081</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D40" s="2">
         <v>1</v>
@@ -1212,7 +1212,7 @@
         <v>3838</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D41" s="2">
         <v>1</v>

</xml_diff>